<commit_message>
fix: INPUT_FILE stock_sample.xlsx로 변경 및 BOM완제품 이름 정상 표시
sku_ro 쿼리에 bundled_sku_ro.sku_id 포함으로 완제품 9개 이름/코드 확인:
- 삼성라이온즈 어린이회원 세트 4종 (7/9/11/13호)
- NCT JNJM BOTH SIDES SET 2종
- EXO REVERXE Big SMini SET
- Jung Seunghwan HOODIE SET
- AHOF LIGHT STICK SET

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stock_ledger_result.xlsx
+++ b/stock_ledger_result.xlsx
@@ -6318,7 +6318,7 @@
         <v>15854</v>
       </c>
       <c r="P87" s="3" t="n">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="Q87" s="3" t="n">
         <v>0</v>
@@ -6385,7 +6385,7 @@
         <v>10913</v>
       </c>
       <c r="P88" s="3" t="n">
-        <v>208</v>
+        <v>277</v>
       </c>
       <c r="Q88" s="3" t="n">
         <v>0</v>
@@ -6452,7 +6452,7 @@
         <v>7963</v>
       </c>
       <c r="P89" s="3" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="Q89" s="3" t="n">
         <v>0</v>
@@ -6519,7 +6519,7 @@
         <v>1196</v>
       </c>
       <c r="P90" s="3" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="Q90" s="3" t="n">
         <v>0</v>
@@ -6586,7 +6586,7 @@
         <v>376</v>
       </c>
       <c r="P91" s="3" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="Q91" s="3" t="n">
         <v>0</v>
@@ -7189,7 +7189,7 @@
         <v>7</v>
       </c>
       <c r="P100" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q100" s="3" t="n">
         <v>0</v>
@@ -7591,7 +7591,7 @@
         <v>0</v>
       </c>
       <c r="P106" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q106" s="3" t="n">
         <v>0</v>
@@ -8261,7 +8261,7 @@
         <v>156</v>
       </c>
       <c r="P116" s="3" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Q116" s="3" t="n">
         <v>0</v>
@@ -8529,7 +8529,7 @@
         <v>11</v>
       </c>
       <c r="P120" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q120" s="3" t="n">
         <v>0</v>
@@ -8663,7 +8663,7 @@
         <v>3</v>
       </c>
       <c r="P122" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q122" s="3" t="n">
         <v>0</v>
@@ -8730,7 +8730,7 @@
         <v>2</v>
       </c>
       <c r="P123" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q123" s="3" t="n">
         <v>0</v>
@@ -9065,7 +9065,7 @@
         <v>10</v>
       </c>
       <c r="P128" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q128" s="3" t="n">
         <v>0</v>
@@ -11159,8 +11159,16 @@
           <t>256402567778945</t>
         </is>
       </c>
-      <c r="C160" s="2" t="inlineStr"/>
-      <c r="D160" s="2" t="inlineStr"/>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>EXO The 8th Album [REVERXE] (Big SMini Ver.)(SMART ALBUM)(B VER.) SET</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>254QEXABREVEBSSET</t>
+        </is>
+      </c>
       <c r="E160" s="2" t="inlineStr"/>
       <c r="F160" s="2" t="inlineStr"/>
       <c r="G160" s="2" t="inlineStr">
@@ -11210,8 +11218,16 @@
           <t>288938109329217</t>
         </is>
       </c>
-      <c r="C161" s="2" t="inlineStr"/>
-      <c r="D161" s="2" t="inlineStr"/>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>NCT JNJM The 1st Mini Album [BOTH SIDES] (EVIDENCE Ver.)(SMART ALBUM) SET</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>261QJJABBOSDSSET</t>
+        </is>
+      </c>
       <c r="E161" s="2" t="inlineStr"/>
       <c r="F161" s="2" t="inlineStr"/>
       <c r="G161" s="2" t="inlineStr">
@@ -14522,7 +14538,7 @@
         <v>1200</v>
       </c>
       <c r="P215" s="3" t="n">
-        <v>825</v>
+        <v>846</v>
       </c>
       <c r="Q215" s="3" t="n">
         <v>0</v>
@@ -14589,7 +14605,7 @@
         <v>15837</v>
       </c>
       <c r="P216" s="3" t="n">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="Q216" s="3" t="n">
         <v>0</v>
@@ -14656,7 +14672,7 @@
         <v>13178</v>
       </c>
       <c r="P217" s="3" t="n">
-        <v>208</v>
+        <v>277</v>
       </c>
       <c r="Q217" s="3" t="n">
         <v>0</v>
@@ -14723,7 +14739,7 @@
         <v>7961</v>
       </c>
       <c r="P218" s="3" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="Q218" s="3" t="n">
         <v>0</v>
@@ -14790,7 +14806,7 @@
         <v>1193</v>
       </c>
       <c r="P219" s="3" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="Q219" s="3" t="n">
         <v>0</v>
@@ -14857,7 +14873,7 @@
         <v>227</v>
       </c>
       <c r="P220" s="3" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="Q220" s="3" t="n">
         <v>0</v>
@@ -14924,7 +14940,7 @@
         <v>374</v>
       </c>
       <c r="P221" s="3" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="Q221" s="3" t="n">
         <v>0</v>
@@ -15527,7 +15543,7 @@
         <v>0</v>
       </c>
       <c r="P230" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q230" s="3" t="n">
         <v>0</v>
@@ -15661,7 +15677,7 @@
         <v>273</v>
       </c>
       <c r="P232" s="3" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="Q232" s="3" t="n">
         <v>0</v>
@@ -15728,7 +15744,7 @@
         <v>800</v>
       </c>
       <c r="P233" s="3" t="n">
-        <v>430</v>
+        <v>480</v>
       </c>
       <c r="Q233" s="3" t="n">
         <v>0</v>
@@ -15795,7 +15811,7 @@
         <v>400</v>
       </c>
       <c r="P234" s="3" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="Q234" s="3" t="n">
         <v>0</v>
@@ -15862,7 +15878,7 @@
         <v>400</v>
       </c>
       <c r="P235" s="3" t="n">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="Q235" s="3" t="n">
         <v>0</v>
@@ -16063,7 +16079,7 @@
         <v>0</v>
       </c>
       <c r="P238" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q238" s="3" t="n">
         <v>0</v>
@@ -16197,7 +16213,7 @@
         <v>0</v>
       </c>
       <c r="P240" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q240" s="3" t="n">
         <v>0</v>
@@ -16264,7 +16280,7 @@
         <v>1</v>
       </c>
       <c r="P241" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q241" s="3" t="n">
         <v>0</v>
@@ -16599,7 +16615,7 @@
         <v>8</v>
       </c>
       <c r="P246" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q246" s="3" t="n">
         <v>0</v>
@@ -18358,8 +18374,16 @@
           <t>256402567778945</t>
         </is>
       </c>
-      <c r="C273" s="2" t="inlineStr"/>
-      <c r="D273" s="2" t="inlineStr"/>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>EXO The 8th Album [REVERXE] (Big SMini Ver.)(SMART ALBUM)(B VER.) SET</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>254QEXABREVEBSSET</t>
+        </is>
+      </c>
       <c r="E273" s="2" t="inlineStr"/>
       <c r="F273" s="2" t="inlineStr"/>
       <c r="G273" s="2" t="inlineStr">
@@ -20028,7 +20052,7 @@
         <v>774</v>
       </c>
       <c r="P301" s="3" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="Q301" s="3" t="n">
         <v>0</v>
@@ -20095,7 +20119,7 @@
         <v>560</v>
       </c>
       <c r="P302" s="3" t="n">
-        <v>825</v>
+        <v>846</v>
       </c>
       <c r="Q302" s="3" t="n">
         <v>0</v>
@@ -20162,7 +20186,7 @@
         <v>15735</v>
       </c>
       <c r="P303" s="3" t="n">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="Q303" s="3" t="n">
         <v>0</v>
@@ -20229,7 +20253,7 @@
         <v>13113</v>
       </c>
       <c r="P304" s="3" t="n">
-        <v>208</v>
+        <v>277</v>
       </c>
       <c r="Q304" s="3" t="n">
         <v>0</v>
@@ -20296,7 +20320,7 @@
         <v>7941</v>
       </c>
       <c r="P305" s="3" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="Q305" s="3" t="n">
         <v>0</v>
@@ -20363,7 +20387,7 @@
         <v>1185</v>
       </c>
       <c r="P306" s="3" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="Q306" s="3" t="n">
         <v>0</v>
@@ -20430,7 +20454,7 @@
         <v>226</v>
       </c>
       <c r="P307" s="3" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="Q307" s="3" t="n">
         <v>0</v>
@@ -20497,7 +20521,7 @@
         <v>373</v>
       </c>
       <c r="P308" s="3" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="Q308" s="3" t="n">
         <v>0</v>
@@ -20765,7 +20789,7 @@
         <v>1304</v>
       </c>
       <c r="P312" s="3" t="n">
-        <v>211</v>
+        <v>316</v>
       </c>
       <c r="Q312" s="3" t="n">
         <v>0</v>
@@ -20832,7 +20856,7 @@
         <v>438</v>
       </c>
       <c r="P313" s="3" t="n">
-        <v>97</v>
+        <v>162</v>
       </c>
       <c r="Q313" s="3" t="n">
         <v>0</v>
@@ -20966,7 +20990,7 @@
         <v>6</v>
       </c>
       <c r="P315" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q315" s="3" t="n">
         <v>0</v>
@@ -21234,7 +21258,7 @@
         <v>0</v>
       </c>
       <c r="P319" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q319" s="3" t="n">
         <v>0</v>
@@ -21301,7 +21325,7 @@
         <v>151</v>
       </c>
       <c r="P320" s="3" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Q320" s="3" t="n">
         <v>0</v>
@@ -21368,7 +21392,7 @@
         <v>271</v>
       </c>
       <c r="P321" s="3" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="Q321" s="3" t="n">
         <v>0</v>
@@ -21435,7 +21459,7 @@
         <v>482</v>
       </c>
       <c r="P322" s="3" t="n">
-        <v>430</v>
+        <v>480</v>
       </c>
       <c r="Q322" s="3" t="n">
         <v>0</v>
@@ -21569,7 +21593,7 @@
         <v>355</v>
       </c>
       <c r="P324" s="3" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="Q324" s="3" t="n">
         <v>0</v>
@@ -21636,7 +21660,7 @@
         <v>343</v>
       </c>
       <c r="P325" s="3" t="n">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="Q325" s="3" t="n">
         <v>0</v>
@@ -23596,8 +23620,16 @@
           <t>292102979684869</t>
         </is>
       </c>
-      <c r="C355" s="2" t="inlineStr"/>
-      <c r="D355" s="2" t="inlineStr"/>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>삼성라이온즈 2026 어린이회원 라온 X 리틀라이언 7호 SET</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>26CL-KD-LL-001-SET</t>
+        </is>
+      </c>
       <c r="E355" s="2" t="inlineStr"/>
       <c r="F355" s="2" t="inlineStr"/>
       <c r="G355" s="2" t="inlineStr">
@@ -23647,8 +23679,16 @@
           <t>292103490903237</t>
         </is>
       </c>
-      <c r="C356" s="2" t="inlineStr"/>
-      <c r="D356" s="2" t="inlineStr"/>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>삼성라이온즈 2026 어린이회원 라온 X 리틀라이언 9호 SET</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>26CL-KD-LL-002-SET</t>
+        </is>
+      </c>
       <c r="E356" s="2" t="inlineStr"/>
       <c r="F356" s="2" t="inlineStr"/>
       <c r="G356" s="2" t="inlineStr">
@@ -23698,8 +23738,16 @@
           <t>292104088054277</t>
         </is>
       </c>
-      <c r="C357" s="2" t="inlineStr"/>
-      <c r="D357" s="2" t="inlineStr"/>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>삼성라이온즈 2026 어린이회원 라온 X 리틀라이언 11호 SET</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>26CL-KD-LL-003-SET</t>
+        </is>
+      </c>
       <c r="E357" s="2" t="inlineStr"/>
       <c r="F357" s="2" t="inlineStr"/>
       <c r="G357" s="2" t="inlineStr">
@@ -23749,8 +23797,16 @@
           <t>292104573467843</t>
         </is>
       </c>
-      <c r="C358" s="2" t="inlineStr"/>
-      <c r="D358" s="2" t="inlineStr"/>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>삼성라이온즈 2026 어린이회원 라온 X 리틀라이언 13호 SET</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>26CL-KD-LL-004-SET</t>
+        </is>
+      </c>
       <c r="E358" s="2" t="inlineStr"/>
       <c r="F358" s="2" t="inlineStr"/>
       <c r="G358" s="2" t="inlineStr">
@@ -30812,7 +30868,7 @@
         <v>762</v>
       </c>
       <c r="P465" s="3" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="Q465" s="3" t="n">
         <v>0</v>
@@ -30879,7 +30935,7 @@
         <v>524</v>
       </c>
       <c r="P466" s="3" t="n">
-        <v>825</v>
+        <v>846</v>
       </c>
       <c r="Q466" s="3" t="n">
         <v>0</v>
@@ -30946,7 +31002,7 @@
         <v>15723</v>
       </c>
       <c r="P467" s="3" t="n">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="Q467" s="3" t="n">
         <v>0</v>
@@ -31013,7 +31069,7 @@
         <v>13100</v>
       </c>
       <c r="P468" s="3" t="n">
-        <v>208</v>
+        <v>277</v>
       </c>
       <c r="Q468" s="3" t="n">
         <v>0</v>
@@ -31080,7 +31136,7 @@
         <v>7939</v>
       </c>
       <c r="P469" s="3" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="Q469" s="3" t="n">
         <v>0</v>
@@ -31147,7 +31203,7 @@
         <v>1183</v>
       </c>
       <c r="P470" s="3" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="Q470" s="3" t="n">
         <v>0</v>
@@ -31214,7 +31270,7 @@
         <v>371</v>
       </c>
       <c r="P471" s="3" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="Q471" s="3" t="n">
         <v>0</v>
@@ -31281,7 +31337,7 @@
         <v>1303</v>
       </c>
       <c r="P472" s="3" t="n">
-        <v>211</v>
+        <v>316</v>
       </c>
       <c r="Q472" s="3" t="n">
         <v>0</v>
@@ -31348,7 +31404,7 @@
         <v>434</v>
       </c>
       <c r="P473" s="3" t="n">
-        <v>97</v>
+        <v>162</v>
       </c>
       <c r="Q473" s="3" t="n">
         <v>0</v>
@@ -31616,7 +31672,7 @@
         <v>150</v>
       </c>
       <c r="P477" s="3" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Q477" s="3" t="n">
         <v>0</v>
@@ -31683,7 +31739,7 @@
         <v>464</v>
       </c>
       <c r="P478" s="3" t="n">
-        <v>430</v>
+        <v>480</v>
       </c>
       <c r="Q478" s="3" t="n">
         <v>0</v>
@@ -31901,8 +31957,16 @@
           <t>248652059610818</t>
         </is>
       </c>
-      <c r="C482" s="2" t="inlineStr"/>
-      <c r="D482" s="2" t="inlineStr"/>
+      <c r="C482" s="2" t="inlineStr">
+        <is>
+          <t>(본품+사은품) 2025 Jung Seunghwan OFFICIAL MD HOODIE</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>SET8809954225420</t>
+        </is>
+      </c>
       <c r="E482" s="2" t="inlineStr"/>
       <c r="F482" s="2" t="inlineStr"/>
       <c r="G482" s="2" t="inlineStr">
@@ -31952,8 +32016,16 @@
           <t>281063542028801</t>
         </is>
       </c>
-      <c r="C483" s="2" t="inlineStr"/>
-      <c r="D483" s="2" t="inlineStr"/>
+      <c r="C483" s="2" t="inlineStr">
+        <is>
+          <t>NCT JNJM The 1st Mini Album [BOTH SIDES] (POSTER Ver.) SET</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>261QJJABBOSDPSSET</t>
+        </is>
+      </c>
       <c r="E483" s="2" t="inlineStr"/>
       <c r="F483" s="2" t="inlineStr"/>
       <c r="G483" s="2" t="inlineStr">
@@ -43367,7 +43439,7 @@
         <v>753</v>
       </c>
       <c r="P666" s="3" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="Q666" s="3" t="n">
         <v>0</v>
@@ -43434,7 +43506,7 @@
         <v>477</v>
       </c>
       <c r="P667" s="3" t="n">
-        <v>825</v>
+        <v>846</v>
       </c>
       <c r="Q667" s="3" t="n">
         <v>0</v>
@@ -43501,7 +43573,7 @@
         <v>15704</v>
       </c>
       <c r="P668" s="3" t="n">
-        <v>264</v>
+        <v>343</v>
       </c>
       <c r="Q668" s="3" t="n">
         <v>0</v>
@@ -43568,7 +43640,7 @@
         <v>13080</v>
       </c>
       <c r="P669" s="3" t="n">
-        <v>208</v>
+        <v>277</v>
       </c>
       <c r="Q669" s="3" t="n">
         <v>0</v>
@@ -43635,7 +43707,7 @@
         <v>7931</v>
       </c>
       <c r="P670" s="3" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="Q670" s="3" t="n">
         <v>0</v>
@@ -43702,7 +43774,7 @@
         <v>1179</v>
       </c>
       <c r="P671" s="3" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="Q671" s="3" t="n">
         <v>0</v>
@@ -43769,7 +43841,7 @@
         <v>1302</v>
       </c>
       <c r="P672" s="3" t="n">
-        <v>211</v>
+        <v>316</v>
       </c>
       <c r="Q672" s="3" t="n">
         <v>0</v>
@@ -43836,7 +43908,7 @@
         <v>432</v>
       </c>
       <c r="P673" s="3" t="n">
-        <v>97</v>
+        <v>162</v>
       </c>
       <c r="Q673" s="3" t="n">
         <v>0</v>
@@ -43970,7 +44042,7 @@
         <v>5</v>
       </c>
       <c r="P675" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q675" s="3" t="n">
         <v>0</v>
@@ -44238,7 +44310,7 @@
         <v>1</v>
       </c>
       <c r="P679" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q679" s="3" t="n">
         <v>0</v>
@@ -44439,7 +44511,7 @@
         <v>1</v>
       </c>
       <c r="P682" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q682" s="3" t="n">
         <v>0</v>
@@ -44640,7 +44712,7 @@
         <v>1</v>
       </c>
       <c r="P685" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q685" s="3" t="n">
         <v>0</v>
@@ -44975,7 +45047,7 @@
         <v>1</v>
       </c>
       <c r="P690" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q690" s="3" t="n">
         <v>0</v>
@@ -45243,7 +45315,7 @@
         <v>149</v>
       </c>
       <c r="P694" s="3" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Q694" s="3" t="n">
         <v>0</v>
@@ -45310,7 +45382,7 @@
         <v>270</v>
       </c>
       <c r="P695" s="3" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="Q695" s="3" t="n">
         <v>0</v>
@@ -45377,7 +45449,7 @@
         <v>3173</v>
       </c>
       <c r="P696" s="3" t="n">
-        <v>430</v>
+        <v>480</v>
       </c>
       <c r="Q696" s="3" t="n">
         <v>0</v>
@@ -45444,7 +45516,7 @@
         <v>352</v>
       </c>
       <c r="P697" s="3" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="Q697" s="3" t="n">
         <v>0</v>
@@ -45511,7 +45583,7 @@
         <v>341</v>
       </c>
       <c r="P698" s="3" t="n">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="Q698" s="3" t="n">
         <v>0</v>
@@ -45578,7 +45650,7 @@
         <v>0</v>
       </c>
       <c r="P699" s="3" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="Q699" s="3" t="n">
         <v>0</v>
@@ -45645,7 +45717,7 @@
         <v>0</v>
       </c>
       <c r="P700" s="3" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="Q700" s="3" t="n">
         <v>0</v>
@@ -45779,7 +45851,7 @@
         <v>1</v>
       </c>
       <c r="P702" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q702" s="3" t="n">
         <v>0</v>
@@ -45913,7 +45985,7 @@
         <v>1</v>
       </c>
       <c r="P704" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q704" s="3" t="n">
         <v>0</v>
@@ -45980,7 +46052,7 @@
         <v>2</v>
       </c>
       <c r="P705" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q705" s="3" t="n">
         <v>0</v>
@@ -46784,7 +46856,7 @@
         <v>1</v>
       </c>
       <c r="P717" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q717" s="3" t="n">
         <v>0</v>
@@ -46985,7 +47057,7 @@
         <v>1</v>
       </c>
       <c r="P720" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q720" s="3" t="n">
         <v>0</v>
@@ -47454,7 +47526,7 @@
         <v>1</v>
       </c>
       <c r="P727" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q727" s="3" t="n">
         <v>0</v>
@@ -47789,7 +47861,7 @@
         <v>10</v>
       </c>
       <c r="P732" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q732" s="3" t="n">
         <v>0</v>
@@ -48057,7 +48129,7 @@
         <v>5</v>
       </c>
       <c r="P736" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q736" s="3" t="n">
         <v>0</v>
@@ -49263,7 +49335,7 @@
         <v>1</v>
       </c>
       <c r="P754" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q754" s="3" t="n">
         <v>0</v>
@@ -49598,7 +49670,7 @@
         <v>1</v>
       </c>
       <c r="P759" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q759" s="3" t="n">
         <v>0</v>
@@ -50670,7 +50742,7 @@
         <v>0</v>
       </c>
       <c r="P775" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q775" s="3" t="n">
         <v>0</v>
@@ -51156,8 +51228,16 @@
           <t>281063542028801</t>
         </is>
       </c>
-      <c r="C783" s="2" t="inlineStr"/>
-      <c r="D783" s="2" t="inlineStr"/>
+      <c r="C783" s="2" t="inlineStr">
+        <is>
+          <t>NCT JNJM The 1st Mini Album [BOTH SIDES] (POSTER Ver.) SET</t>
+        </is>
+      </c>
+      <c r="D783" s="2" t="inlineStr">
+        <is>
+          <t>261QJJABBOSDPSSET</t>
+        </is>
+      </c>
       <c r="E783" s="2" t="inlineStr"/>
       <c r="F783" s="2" t="inlineStr"/>
       <c r="G783" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: sku_nm 누락 SKU를 delivery_item_ro.item_name으로 보완
sku_ro에서 완전 삭제된 72개 SKU 중 delivery_item_ro에 item_name이 있는
25개는 자동으로 이름 채움. 나머지 47개는 샘플 데이터 어디에도 이름 없음.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stock_ledger_result.xlsx
+++ b/stock_ledger_result.xlsx
@@ -11277,7 +11277,11 @@
           <t>193630013852160</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr"/>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR OFFICIAL FANLIGHT Special Edition</t>
+        </is>
+      </c>
       <c r="D162" s="2" t="inlineStr"/>
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr"/>
@@ -11324,7 +11328,11 @@
           <t>193630014302720</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr"/>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>aespa OFFICIAL FANLIGHT VER.2</t>
+        </is>
+      </c>
       <c r="D163" s="2" t="inlineStr"/>
       <c r="E163" s="2" t="inlineStr"/>
       <c r="F163" s="2" t="inlineStr"/>
@@ -11418,7 +11426,11 @@
           <t>193630015506944</t>
         </is>
       </c>
-      <c r="C165" s="2" t="inlineStr"/>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Red Velvet OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D165" s="2" t="inlineStr"/>
       <c r="E165" s="2" t="inlineStr"/>
       <c r="F165" s="2" t="inlineStr"/>
@@ -11465,7 +11477,11 @@
           <t>193630015891968</t>
         </is>
       </c>
-      <c r="C166" s="2" t="inlineStr"/>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>NCT DREAM OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D166" s="2" t="inlineStr"/>
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr"/>
@@ -11559,7 +11575,11 @@
           <t>193630016276992</t>
         </is>
       </c>
-      <c r="C168" s="2" t="inlineStr"/>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D168" s="2" t="inlineStr"/>
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr"/>
@@ -11653,7 +11673,11 @@
           <t>193630048348672</t>
         </is>
       </c>
-      <c r="C170" s="2" t="inlineStr"/>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>RIIZE The 1st Album [ODYSSEY] (Midnight Mirage A Ver.)(SMART ALBUM)</t>
+        </is>
+      </c>
       <c r="D170" s="2" t="inlineStr"/>
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr"/>
@@ -11700,7 +11724,11 @@
           <t>193630053272064</t>
         </is>
       </c>
-      <c r="C171" s="2" t="inlineStr"/>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH Single Album [WISH] (WICHU Ver.)(SMART ALBUM)</t>
+        </is>
+      </c>
       <c r="D171" s="2" t="inlineStr"/>
       <c r="E171" s="2" t="inlineStr"/>
       <c r="F171" s="2" t="inlineStr"/>
@@ -11888,7 +11916,11 @@
           <t>193630118185472</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr"/>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH MINI FANLIGHT KEYRING VER. 2.0</t>
+        </is>
+      </c>
       <c r="D175" s="2" t="inlineStr"/>
       <c r="E175" s="2" t="inlineStr"/>
       <c r="F175" s="2" t="inlineStr"/>
@@ -11935,7 +11967,11 @@
           <t>203219200682560</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr"/>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>NCT Fansignal Lip Balm</t>
+        </is>
+      </c>
       <c r="D176" s="2" t="inlineStr"/>
       <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr"/>
@@ -11982,7 +12018,11 @@
           <t>204095535711360</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr"/>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Fansignal Lip Balm 비즈스트랩 NCT</t>
+        </is>
+      </c>
       <c r="D177" s="2" t="inlineStr"/>
       <c r="E177" s="2" t="inlineStr"/>
       <c r="F177" s="2" t="inlineStr"/>
@@ -18433,7 +18473,11 @@
           <t>193630013852160</t>
         </is>
       </c>
-      <c r="C274" s="2" t="inlineStr"/>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR OFFICIAL FANLIGHT Special Edition</t>
+        </is>
+      </c>
       <c r="D274" s="2" t="inlineStr"/>
       <c r="E274" s="2" t="inlineStr"/>
       <c r="F274" s="2" t="inlineStr"/>
@@ -18480,7 +18524,11 @@
           <t>193630015703552</t>
         </is>
       </c>
-      <c r="C275" s="2" t="inlineStr"/>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>NCT 127 OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D275" s="2" t="inlineStr"/>
       <c r="E275" s="2" t="inlineStr"/>
       <c r="F275" s="2" t="inlineStr"/>
@@ -18527,7 +18575,11 @@
           <t>193630015891968</t>
         </is>
       </c>
-      <c r="C276" s="2" t="inlineStr"/>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>NCT DREAM OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D276" s="2" t="inlineStr"/>
       <c r="E276" s="2" t="inlineStr"/>
       <c r="F276" s="2" t="inlineStr"/>
@@ -18574,7 +18626,11 @@
           <t>193630016276992</t>
         </is>
       </c>
-      <c r="C277" s="2" t="inlineStr"/>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D277" s="2" t="inlineStr"/>
       <c r="E277" s="2" t="inlineStr"/>
       <c r="F277" s="2" t="inlineStr"/>
@@ -18621,7 +18677,11 @@
           <t>193630020512256</t>
         </is>
       </c>
-      <c r="C278" s="2" t="inlineStr"/>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>STYLE - STYLING SET</t>
+        </is>
+      </c>
       <c r="D278" s="2" t="inlineStr"/>
       <c r="E278" s="2" t="inlineStr"/>
       <c r="F278" s="2" t="inlineStr"/>
@@ -18668,7 +18728,11 @@
           <t>193630041319936</t>
         </is>
       </c>
-      <c r="C279" s="2" t="inlineStr"/>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>The Chase - BEADS STRAP SET [JIWOO]</t>
+        </is>
+      </c>
       <c r="D279" s="2" t="inlineStr"/>
       <c r="E279" s="2" t="inlineStr"/>
       <c r="F279" s="2" t="inlineStr"/>
@@ -18715,7 +18779,11 @@
           <t>193630042753536</t>
         </is>
       </c>
-      <c r="C280" s="2" t="inlineStr"/>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>The Chase - 4X6 PHOTO SET</t>
+        </is>
+      </c>
       <c r="D280" s="2" t="inlineStr"/>
       <c r="E280" s="2" t="inlineStr"/>
       <c r="F280" s="2" t="inlineStr"/>
@@ -18762,7 +18830,11 @@
           <t>193630048938496</t>
         </is>
       </c>
-      <c r="C281" s="2" t="inlineStr"/>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR The 12th Album [Super Junior25] (PHOTOBOOK Ver.)</t>
+        </is>
+      </c>
       <c r="D281" s="2" t="inlineStr"/>
       <c r="E281" s="2" t="inlineStr"/>
       <c r="F281" s="2" t="inlineStr"/>
@@ -18809,7 +18881,11 @@
           <t>193630049102336</t>
         </is>
       </c>
-      <c r="C282" s="2" t="inlineStr"/>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR The 12th Album [Super Junior25] (SMini Ver.)(SMART ALBUM)</t>
+        </is>
+      </c>
       <c r="D282" s="2" t="inlineStr"/>
       <c r="E282" s="2" t="inlineStr"/>
       <c r="F282" s="2" t="inlineStr"/>
@@ -18856,7 +18932,11 @@
           <t>193630210476544</t>
         </is>
       </c>
-      <c r="C283" s="2" t="inlineStr"/>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>2025 RIIZE CONCERT TOUR [RIIZING LOUD] LITTLE RIIZE T-SHIRT [SOHEE]</t>
+        </is>
+      </c>
       <c r="D283" s="2" t="inlineStr"/>
       <c r="E283" s="2" t="inlineStr"/>
       <c r="F283" s="2" t="inlineStr"/>
@@ -18903,7 +18983,11 @@
           <t>214641095461824</t>
         </is>
       </c>
-      <c r="C284" s="2" t="inlineStr"/>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>FOCUS - POSTER SET [JIWOO]</t>
+        </is>
+      </c>
       <c r="D284" s="2" t="inlineStr"/>
       <c r="E284" s="2" t="inlineStr"/>
       <c r="F284" s="2" t="inlineStr"/>
@@ -18950,7 +19034,11 @@
           <t>214641096043456</t>
         </is>
       </c>
-      <c r="C285" s="2" t="inlineStr"/>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>FOCUS - RANDOM TRADING CARD A VER.</t>
+        </is>
+      </c>
       <c r="D285" s="2" t="inlineStr"/>
       <c r="E285" s="2" t="inlineStr"/>
       <c r="F285" s="2" t="inlineStr"/>
@@ -23856,7 +23944,11 @@
           <t>193630013852160</t>
         </is>
       </c>
-      <c r="C359" s="2" t="inlineStr"/>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR OFFICIAL FANLIGHT Special Edition</t>
+        </is>
+      </c>
       <c r="D359" s="2" t="inlineStr"/>
       <c r="E359" s="2" t="inlineStr"/>
       <c r="F359" s="2" t="inlineStr"/>
@@ -23903,7 +23995,11 @@
           <t>193630014302720</t>
         </is>
       </c>
-      <c r="C360" s="2" t="inlineStr"/>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>aespa OFFICIAL FANLIGHT VER.2</t>
+        </is>
+      </c>
       <c r="D360" s="2" t="inlineStr"/>
       <c r="E360" s="2" t="inlineStr"/>
       <c r="F360" s="2" t="inlineStr"/>
@@ -23950,7 +24046,11 @@
           <t>193630014704128</t>
         </is>
       </c>
-      <c r="C361" s="2" t="inlineStr"/>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>TVXQ! OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D361" s="2" t="inlineStr"/>
       <c r="E361" s="2" t="inlineStr"/>
       <c r="F361" s="2" t="inlineStr"/>
@@ -23997,7 +24097,11 @@
           <t>193630015506944</t>
         </is>
       </c>
-      <c r="C362" s="2" t="inlineStr"/>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>Red Velvet OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D362" s="2" t="inlineStr"/>
       <c r="E362" s="2" t="inlineStr"/>
       <c r="F362" s="2" t="inlineStr"/>
@@ -24044,7 +24148,11 @@
           <t>193630016276992</t>
         </is>
       </c>
-      <c r="C363" s="2" t="inlineStr"/>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D363" s="2" t="inlineStr"/>
       <c r="E363" s="2" t="inlineStr"/>
       <c r="F363" s="2" t="inlineStr"/>
@@ -24091,7 +24199,11 @@
           <t>193630053272064</t>
         </is>
       </c>
-      <c r="C364" s="2" t="inlineStr"/>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH Single Album [WISH] (WICHU Ver.)(SMART ALBUM)</t>
+        </is>
+      </c>
       <c r="D364" s="2" t="inlineStr"/>
       <c r="E364" s="2" t="inlineStr"/>
       <c r="F364" s="2" t="inlineStr"/>
@@ -24138,7 +24250,11 @@
           <t>193630206511616</t>
         </is>
       </c>
-      <c r="C365" s="2" t="inlineStr"/>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>2025 RIIZE CONCERT TOUR [RIIZING LOUD] TRACK JACKET SET [ANTON]</t>
+        </is>
+      </c>
       <c r="D365" s="2" t="inlineStr"/>
       <c r="E365" s="2" t="inlineStr"/>
       <c r="F365" s="2" t="inlineStr"/>
@@ -32075,7 +32191,11 @@
           <t>193630013852160</t>
         </is>
       </c>
-      <c r="C484" s="2" t="inlineStr"/>
+      <c r="C484" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR OFFICIAL FANLIGHT Special Edition</t>
+        </is>
+      </c>
       <c r="D484" s="2" t="inlineStr"/>
       <c r="E484" s="2" t="inlineStr"/>
       <c r="F484" s="2" t="inlineStr"/>
@@ -32122,7 +32242,11 @@
           <t>193630015891968</t>
         </is>
       </c>
-      <c r="C485" s="2" t="inlineStr"/>
+      <c r="C485" s="2" t="inlineStr">
+        <is>
+          <t>NCT DREAM OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D485" s="2" t="inlineStr"/>
       <c r="E485" s="2" t="inlineStr"/>
       <c r="F485" s="2" t="inlineStr"/>
@@ -32169,7 +32293,11 @@
           <t>193630016276992</t>
         </is>
       </c>
-      <c r="C486" s="2" t="inlineStr"/>
+      <c r="C486" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D486" s="2" t="inlineStr"/>
       <c r="E486" s="2" t="inlineStr"/>
       <c r="F486" s="2" t="inlineStr"/>
@@ -32216,7 +32344,11 @@
           <t>193630048938496</t>
         </is>
       </c>
-      <c r="C487" s="2" t="inlineStr"/>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR The 12th Album [Super Junior25] (PHOTOBOOK Ver.)</t>
+        </is>
+      </c>
       <c r="D487" s="2" t="inlineStr"/>
       <c r="E487" s="2" t="inlineStr"/>
       <c r="F487" s="2" t="inlineStr"/>
@@ -32310,7 +32442,11 @@
           <t>193630065486336</t>
         </is>
       </c>
-      <c r="C489" s="2" t="inlineStr"/>
+      <c r="C489" s="2" t="inlineStr">
+        <is>
+          <t>NCT DREAM [DREAMSCAPE] (DREAMSCAPE Ver.)</t>
+        </is>
+      </c>
       <c r="D489" s="2" t="inlineStr"/>
       <c r="E489" s="2" t="inlineStr"/>
       <c r="F489" s="2" t="inlineStr"/>
@@ -32404,7 +32540,11 @@
           <t>193630070245888</t>
         </is>
       </c>
-      <c r="C491" s="2" t="inlineStr"/>
+      <c r="C491" s="2" t="inlineStr">
+        <is>
+          <t>aespa The 6th Mini Album [Rich Man] (RICH MAN BAG Ver.)</t>
+        </is>
+      </c>
       <c r="D491" s="2" t="inlineStr"/>
       <c r="E491" s="2" t="inlineStr"/>
       <c r="F491" s="2" t="inlineStr"/>
@@ -33438,7 +33578,11 @@
           <t>203219200682560</t>
         </is>
       </c>
-      <c r="C513" s="2" t="inlineStr"/>
+      <c r="C513" s="2" t="inlineStr">
+        <is>
+          <t>NCT Fansignal Lip Balm</t>
+        </is>
+      </c>
       <c r="D513" s="2" t="inlineStr"/>
       <c r="E513" s="2" t="inlineStr"/>
       <c r="F513" s="2" t="inlineStr"/>
@@ -33579,7 +33723,11 @@
           <t>204095535711360</t>
         </is>
       </c>
-      <c r="C516" s="2" t="inlineStr"/>
+      <c r="C516" s="2" t="inlineStr">
+        <is>
+          <t>Fansignal Lip Balm 비즈스트랩 NCT</t>
+        </is>
+      </c>
       <c r="D516" s="2" t="inlineStr"/>
       <c r="E516" s="2" t="inlineStr"/>
       <c r="F516" s="2" t="inlineStr"/>
@@ -51287,7 +51435,11 @@
           <t>193630013852160</t>
         </is>
       </c>
-      <c r="C784" s="2" t="inlineStr"/>
+      <c r="C784" s="2" t="inlineStr">
+        <is>
+          <t>SUPER JUNIOR OFFICIAL FANLIGHT Special Edition</t>
+        </is>
+      </c>
       <c r="D784" s="2" t="inlineStr"/>
       <c r="E784" s="2" t="inlineStr"/>
       <c r="F784" s="2" t="inlineStr"/>
@@ -51334,7 +51486,11 @@
           <t>193630014302720</t>
         </is>
       </c>
-      <c r="C785" s="2" t="inlineStr"/>
+      <c r="C785" s="2" t="inlineStr">
+        <is>
+          <t>aespa OFFICIAL FANLIGHT VER.2</t>
+        </is>
+      </c>
       <c r="D785" s="2" t="inlineStr"/>
       <c r="E785" s="2" t="inlineStr"/>
       <c r="F785" s="2" t="inlineStr"/>
@@ -51428,7 +51584,11 @@
           <t>193630015891968</t>
         </is>
       </c>
-      <c r="C787" s="2" t="inlineStr"/>
+      <c r="C787" s="2" t="inlineStr">
+        <is>
+          <t>NCT DREAM OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D787" s="2" t="inlineStr"/>
       <c r="E787" s="2" t="inlineStr"/>
       <c r="F787" s="2" t="inlineStr"/>
@@ -51475,7 +51635,11 @@
           <t>193630016276992</t>
         </is>
       </c>
-      <c r="C788" s="2" t="inlineStr"/>
+      <c r="C788" s="2" t="inlineStr">
+        <is>
+          <t>NCT WISH OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D788" s="2" t="inlineStr"/>
       <c r="E788" s="2" t="inlineStr"/>
       <c r="F788" s="2" t="inlineStr"/>
@@ -51522,7 +51686,11 @@
           <t>193630048348672</t>
         </is>
       </c>
-      <c r="C789" s="2" t="inlineStr"/>
+      <c r="C789" s="2" t="inlineStr">
+        <is>
+          <t>RIIZE The 1st Album [ODYSSEY] (Midnight Mirage A Ver.)(SMART ALBUM)</t>
+        </is>
+      </c>
       <c r="D789" s="2" t="inlineStr"/>
       <c r="E789" s="2" t="inlineStr"/>
       <c r="F789" s="2" t="inlineStr"/>
@@ -51710,7 +51878,11 @@
           <t>193630120569344</t>
         </is>
       </c>
-      <c r="C793" s="2" t="inlineStr"/>
+      <c r="C793" s="2" t="inlineStr">
+        <is>
+          <t>RIIZE  2025 SEASON'S GREETINGS PHOTO PACK [SHOTARO]</t>
+        </is>
+      </c>
       <c r="D793" s="2" t="inlineStr"/>
       <c r="E793" s="2" t="inlineStr"/>
       <c r="F793" s="2" t="inlineStr"/>
@@ -51898,7 +52070,11 @@
           <t>228137065389248</t>
         </is>
       </c>
-      <c r="C797" s="2" t="inlineStr"/>
+      <c r="C797" s="2" t="inlineStr">
+        <is>
+          <t>RIIZE 2024 PINK CHRISTMAS PHOTO CARD RANDOM PACK</t>
+        </is>
+      </c>
       <c r="D797" s="2" t="inlineStr"/>
       <c r="E797" s="2" t="inlineStr"/>
       <c r="F797" s="2" t="inlineStr"/>
@@ -55275,7 +55451,11 @@
           <t>193630015891968</t>
         </is>
       </c>
-      <c r="C848" s="2" t="inlineStr"/>
+      <c r="C848" s="2" t="inlineStr">
+        <is>
+          <t>NCT DREAM OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D848" s="2" t="inlineStr"/>
       <c r="E848" s="2" t="inlineStr"/>
       <c r="F848" s="2" t="inlineStr"/>
@@ -58163,7 +58343,11 @@
           <t>193630015891968</t>
         </is>
       </c>
-      <c r="C892" s="2" t="inlineStr"/>
+      <c r="C892" s="2" t="inlineStr">
+        <is>
+          <t>NCT DREAM OFFICIAL FANLIGHT</t>
+        </is>
+      </c>
       <c r="D892" s="2" t="inlineStr"/>
       <c r="E892" s="2" t="inlineStr"/>
       <c r="F892" s="2" t="inlineStr"/>

</xml_diff>